<commit_message>
more data, thats it, no logic update
</commit_message>
<xml_diff>
--- a/backend/data-filtering/harbourline_fromcst_dn.xlsx
+++ b/backend/data-filtering/harbourline_fromcst_dn.xlsx
@@ -3983,10 +3983,10 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">

</xml_diff>